<commit_message>
feat: botão limpar base clientes + modelo sem linha exemplo
</commit_message>
<xml_diff>
--- a/public/modelo-base-clientes.xlsx
+++ b/public/modelo-base-clientes.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -427,29 +427,9 @@
         <v>Número Ordem/OS</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>João Silva</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Empresa Exemplo Ltda</v>
-      </c>
-      <c r="C2" t="str">
-        <v>12.345.678/0001-99</v>
-      </c>
-      <c r="D2" t="str">
-        <v>47999990001</v>
-      </c>
-      <c r="E2" t="str">
-        <v>47999990002</v>
-      </c>
-      <c r="F2" t="str">
-        <v>1-1234567890123</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: coluna G Mes Gross manual na base clientes para agrupar no Ajustes
</commit_message>
<xml_diff>
--- a/public/modelo-base-clientes.xlsx
+++ b/public/modelo-base-clientes.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -405,6 +405,7 @@
     <col min="4" max="4" width="28.83203125" customWidth="1"/>
     <col min="5" max="5" width="25.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,10 +427,13 @@
       <c r="F1" t="str">
         <v>Número Ordem/OS</v>
       </c>
+      <c r="G1" t="str">
+        <v>Mês Gross</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>